<commit_message>
Migrate LSA Undergraduate page and prepare all pages for DA
- audience-landing: add /lsa/prospective-students/undergraduate with
  stat-tile cards, two-column text|image columns, foreground-portrait
  hero (image-left/theme-light) and text-right background hero
- hero parser: always emit image + text rows so positional config rows
  line up on document-authored (DA) pages
- cleanup: drop third-party tracking pixels, flatten the live events feed
- academics-directory: rebuild the majors-minors program list as a table block
- recreate missing import-about.js / columns-about.js from the About bundle
- homepage: map the re-authored live hero section
- point URL lists at the live site (imports run from saved snapshots)
- add build-da-docs.mjs + upload-to-da.sh for DA conversion and upload

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-academics-directory.report.xlsx
+++ b/tools/importer/reports/import-academics-directory.report.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="132" uniqueCount="77">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="187" uniqueCount="107">
   <si>
     <t>_reportFile</t>
   </si>
@@ -46,10 +46,34 @@
     <t>url</t>
   </si>
   <si>
+    <t>cgis.report.json</t>
+  </si>
+  <si>
+    <t>[]</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t>cgis</t>
+  </si>
+  <si>
+    <t>success</t>
+  </si>
+  <si>
+    <t>department-landing</t>
+  </si>
+  <si>
+    <t>2026-10-07T15:51:15.956Z</t>
+  </si>
+  <si>
+    <t>Center for Global and Intercultural Study | U-M LSA</t>
+  </si>
+  <si>
+    <t>https://lsa.umich.edu/cgis</t>
+  </si>
+  <si>
     <t>header-footer-source.html.report.json</t>
-  </si>
-  <si>
-    <t/>
   </si>
   <si>
     <t xml:space="preserve">page.evaluate: Error: Failed to import page: Cannot read properties of undefined (reading 'replace')
@@ -85,9 +109,6 @@
     <t>home</t>
   </si>
   <si>
-    <t>success</t>
-  </si>
-  <si>
     <t>homepage</t>
   </si>
   <si>
@@ -103,13 +124,16 @@
     <t>index.report.json</t>
   </si>
   <si>
+    <t>["hero","hero","cards","cards","cards","cards","cards","columns"]</t>
+  </si>
+  <si>
     <t>index</t>
   </si>
   <si>
-    <t>2026-08-13T19:09:49.009Z</t>
-  </si>
-  <si>
-    <t>http://localhost:8082/</t>
+    <t>2026-10-07T15:50:42.735Z</t>
+  </si>
+  <si>
+    <t>https://lsa.umich.edu/</t>
   </si>
   <si>
     <t>rc.report.json</t>
@@ -124,13 +148,13 @@
     <t>unit-home</t>
   </si>
   <si>
-    <t>2026-08-14T14:54:44.130Z</t>
+    <t>2026-10-07T15:51:04.207Z</t>
   </si>
   <si>
     <t>Residential College | U-M LSA</t>
   </si>
   <si>
-    <t>http://localhost:8082/rc.html</t>
+    <t>https://lsa.umich.edu/rc</t>
   </si>
   <si>
     <t>en/footer.report.json</t>
@@ -142,7 +166,7 @@
     <t>en/footer</t>
   </si>
   <si>
-    <t>2026-08-13T18:11:43.199Z</t>
+    <t>2026-10-07T15:47:50.687Z</t>
   </si>
   <si>
     <t>en/nav.report.json</t>
@@ -154,7 +178,7 @@
     <t>en/nav</t>
   </si>
   <si>
-    <t>2026-08-13T18:11:39.386Z</t>
+    <t>2026-10-07T15:47:46.487Z</t>
   </si>
   <si>
     <t>english/undergraduate.report.json</t>
@@ -166,16 +190,34 @@
     <t>english/undergraduate</t>
   </si>
   <si>
-    <t>department-landing</t>
-  </si>
-  <si>
-    <t>2026-08-14T15:34:11.176Z</t>
+    <t>2026-10-07T15:51:08.681Z</t>
   </si>
   <si>
     <t>Undergraduate Students | U-M LSA English Language and Literature</t>
   </si>
   <si>
-    <t>http://localhost:8082/english/undergraduate.html</t>
+    <t>https://lsa.umich.edu/english/undergraduate.html</t>
+  </si>
+  <si>
+    <t>lsa/about.report.json</t>
+  </si>
+  <si>
+    <t>["hero","columns","columns","columns","columns","columns","cards"]</t>
+  </si>
+  <si>
+    <t>lsa/about</t>
+  </si>
+  <si>
+    <t>about</t>
+  </si>
+  <si>
+    <t>2026-10-07T15:50:52.238Z</t>
+  </si>
+  <si>
+    <t>About | U-M LSA U-M College of LSA</t>
+  </si>
+  <si>
+    <t>https://lsa.umich.edu/lsa/about.html</t>
   </si>
   <si>
     <t>lsa/prospective-students.report.json</t>
@@ -190,13 +232,28 @@
     <t>audience-landing</t>
   </si>
   <si>
-    <t>2026-08-13T19:09:54.180Z</t>
+    <t>2026-10-07T15:50:46.629Z</t>
   </si>
   <si>
     <t>Prospective Students | U-M LSA U-M College of LSA</t>
   </si>
   <si>
-    <t>http://localhost:8082/lsa/prospective-students.html</t>
+    <t>https://lsa.umich.edu/lsa/prospective-students.html</t>
+  </si>
+  <si>
+    <t>urop/prospective-students.report.json</t>
+  </si>
+  <si>
+    <t>urop/prospective-students</t>
+  </si>
+  <si>
+    <t>2026-10-07T15:51:10.836Z</t>
+  </si>
+  <si>
+    <t>Prospective UROP Students | U-M LSA UROP: A Center for Research, Scholarship, and Creative Inquiry</t>
+  </si>
+  <si>
+    <t>https://lsa.umich.edu/urop/prospective-students.html</t>
   </si>
   <si>
     <t>lsa/academics/departments-and-units.html.report.json</t>
@@ -227,34 +284,67 @@
     <t>lsa/academics/departments-and-units.report.json</t>
   </si>
   <si>
-    <t>[]</t>
-  </si>
-  <si>
     <t>lsa/academics/departments-and-units</t>
   </si>
   <si>
     <t>academics-listing</t>
   </si>
   <si>
-    <t>2026-08-14T15:34:16.482Z</t>
+    <t>2026-10-07T15:52:40.889Z</t>
   </si>
   <si>
     <t>Departments and Units | U-M LSA U-M College of LSA</t>
   </si>
   <si>
+    <t>https://lsa.umich.edu/lsa/academics/departments-and-units.html</t>
+  </si>
+  <si>
     <t>lsa/academics/majors-minors.report.json</t>
   </si>
   <si>
     <t>lsa/academics/majors-minors</t>
   </si>
   <si>
-    <t>2026-08-13T18:48:55.438Z</t>
+    <t>2026-10-07T15:52:38.323Z</t>
   </si>
   <si>
     <t>Majors and Minors | U-M LSA U-M College of LSA</t>
   </si>
   <si>
-    <t>http://localhost:8082/lsa/academics/majors-minors.html</t>
+    <t>https://lsa.umich.edu/lsa/academics/majors-minors.html</t>
+  </si>
+  <si>
+    <t>lsa/prospective-students/undergraduate.report.json</t>
+  </si>
+  <si>
+    <t>["hero","hero","cards","cards","columns"]</t>
+  </si>
+  <si>
+    <t>lsa/prospective-students/undergraduate</t>
+  </si>
+  <si>
+    <t>2026-10-07T15:50:48.803Z</t>
+  </si>
+  <si>
+    <t>Undergraduate | U-M LSA U-M College of LSA</t>
+  </si>
+  <si>
+    <t>https://lsa.umich.edu/lsa/prospective-students/undergraduate.html</t>
+  </si>
+  <si>
+    <t>psych/prospective-students/undergraduate.report.json</t>
+  </si>
+  <si>
+    <t>psych/prospective-students/undergraduate</t>
+  </si>
+  <si>
+    <t>2026-10-07T15:51:13.626Z</t>
+  </si>
+  <si>
+    <t>Undergraduate | U-M LSA Department of Psychology</t>
+  </si>
+  <si>
+    <t>https://lsa.umich.edu/psych/prospective-students/undergraduate.html</t>
   </si>
 </sst>
 </file>
@@ -643,7 +733,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:K12"/>
+  <dimension ref="A1:K17"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="4" width="50" customWidth="1"/>
@@ -700,60 +790,60 @@
         <v>13</v>
       </c>
       <c r="D2" t="s">
+        <v>13</v>
+      </c>
+      <c r="E2" t="s">
+        <v>13</v>
+      </c>
+      <c r="F2" t="s">
         <v>14</v>
       </c>
-      <c r="E2" t="s">
-        <v>12</v>
-      </c>
-      <c r="F2" t="s">
+      <c r="G2" t="s">
         <v>15</v>
       </c>
-      <c r="G2" t="s">
+      <c r="H2" t="s">
         <v>16</v>
-      </c>
-      <c r="H2" t="s">
-        <v>12</v>
       </c>
       <c r="I2" t="s">
         <v>17</v>
       </c>
       <c r="J2" t="s">
-        <v>12</v>
+        <v>18</v>
       </c>
       <c r="K2" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B3" t="s">
-        <v>20</v>
+        <v>13</v>
       </c>
       <c r="C3" t="s">
-        <v>12</v>
+        <v>21</v>
       </c>
       <c r="D3" t="s">
-        <v>12</v>
+        <v>22</v>
       </c>
       <c r="E3" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="F3" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="G3" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="H3" t="s">
-        <v>23</v>
+        <v>13</v>
       </c>
       <c r="I3" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="J3" t="s">
-        <v>25</v>
+        <v>13</v>
       </c>
       <c r="K3" t="s">
         <v>26</v>
@@ -764,200 +854,200 @@
         <v>27</v>
       </c>
       <c r="B4" t="s">
-        <v>20</v>
+        <v>28</v>
       </c>
       <c r="C4" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="D4" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E4" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="F4" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="G4" t="s">
-        <v>22</v>
+        <v>15</v>
       </c>
       <c r="H4" t="s">
-        <v>23</v>
+        <v>30</v>
       </c>
       <c r="I4" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="J4" t="s">
-        <v>25</v>
+        <v>32</v>
       </c>
       <c r="K4" t="s">
-        <v>30</v>
+        <v>33</v>
       </c>
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="B5" t="s">
+        <v>35</v>
+      </c>
+      <c r="C5" t="s">
+        <v>13</v>
+      </c>
+      <c r="D5" t="s">
+        <v>13</v>
+      </c>
+      <c r="E5" t="s">
+        <v>13</v>
+      </c>
+      <c r="F5" t="s">
+        <v>36</v>
+      </c>
+      <c r="G5" t="s">
+        <v>15</v>
+      </c>
+      <c r="H5" t="s">
+        <v>30</v>
+      </c>
+      <c r="I5" t="s">
+        <v>37</v>
+      </c>
+      <c r="J5" t="s">
         <v>32</v>
       </c>
-      <c r="C5" t="s">
-        <v>12</v>
-      </c>
-      <c r="D5" t="s">
-        <v>12</v>
-      </c>
-      <c r="E5" t="s">
-        <v>12</v>
-      </c>
-      <c r="F5" t="s">
-        <v>33</v>
-      </c>
-      <c r="G5" t="s">
-        <v>22</v>
-      </c>
-      <c r="H5" t="s">
-        <v>34</v>
-      </c>
-      <c r="I5" t="s">
-        <v>35</v>
-      </c>
-      <c r="J5" t="s">
-        <v>36</v>
-      </c>
       <c r="K5" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B6" t="s">
-        <v>12</v>
+        <v>40</v>
       </c>
       <c r="C6" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="D6" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E6" t="s">
-        <v>39</v>
+        <v>13</v>
       </c>
       <c r="F6" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="G6" t="s">
-        <v>22</v>
+        <v>15</v>
       </c>
       <c r="H6" t="s">
-        <v>12</v>
+        <v>42</v>
       </c>
       <c r="I6" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="J6" t="s">
-        <v>12</v>
+        <v>44</v>
       </c>
       <c r="K6" t="s">
-        <v>18</v>
+        <v>45</v>
       </c>
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>42</v>
+        <v>46</v>
       </c>
       <c r="B7" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C7" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="D7" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E7" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="F7" t="s">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="G7" t="s">
-        <v>22</v>
+        <v>15</v>
       </c>
       <c r="H7" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="I7" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="J7" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="K7" t="s">
-        <v>18</v>
+        <v>38</v>
       </c>
     </row>
     <row r="8" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>46</v>
+        <v>50</v>
       </c>
       <c r="B8" t="s">
-        <v>47</v>
+        <v>13</v>
       </c>
       <c r="C8" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="D8" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E8" t="s">
-        <v>12</v>
+        <v>51</v>
       </c>
       <c r="F8" t="s">
-        <v>48</v>
+        <v>52</v>
       </c>
       <c r="G8" t="s">
-        <v>22</v>
+        <v>15</v>
       </c>
       <c r="H8" t="s">
-        <v>49</v>
+        <v>13</v>
       </c>
       <c r="I8" t="s">
-        <v>50</v>
+        <v>53</v>
       </c>
       <c r="J8" t="s">
-        <v>51</v>
+        <v>13</v>
       </c>
       <c r="K8" t="s">
-        <v>52</v>
+        <v>38</v>
       </c>
     </row>
     <row r="9" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="B9" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="C9" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="D9" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E9" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="F9" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="G9" t="s">
-        <v>22</v>
+        <v>15</v>
       </c>
       <c r="H9" t="s">
-        <v>56</v>
+        <v>16</v>
       </c>
       <c r="I9" t="s">
         <v>57</v>
@@ -974,104 +1064,279 @@
         <v>60</v>
       </c>
       <c r="B10" t="s">
-        <v>12</v>
+        <v>61</v>
       </c>
       <c r="C10" t="s">
-        <v>61</v>
+        <v>13</v>
       </c>
       <c r="D10" t="s">
+        <v>13</v>
+      </c>
+      <c r="E10" t="s">
+        <v>13</v>
+      </c>
+      <c r="F10" t="s">
         <v>62</v>
       </c>
-      <c r="E10" t="s">
-        <v>12</v>
-      </c>
-      <c r="F10" t="s">
+      <c r="G10" t="s">
+        <v>15</v>
+      </c>
+      <c r="H10" t="s">
         <v>63</v>
-      </c>
-      <c r="G10" t="s">
-        <v>16</v>
-      </c>
-      <c r="H10" t="s">
-        <v>12</v>
       </c>
       <c r="I10" t="s">
         <v>64</v>
       </c>
       <c r="J10" t="s">
-        <v>12</v>
+        <v>65</v>
       </c>
       <c r="K10" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
     </row>
     <row r="11" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="B11" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="C11" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="D11" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E11" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="F11" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="G11" t="s">
-        <v>22</v>
+        <v>15</v>
       </c>
       <c r="H11" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="I11" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="J11" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="K11" t="s">
-        <v>65</v>
+        <v>73</v>
       </c>
     </row>
     <row r="12" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="B12" t="s">
-        <v>67</v>
+        <v>12</v>
       </c>
       <c r="C12" t="s">
+        <v>13</v>
+      </c>
+      <c r="D12" t="s">
+        <v>13</v>
+      </c>
+      <c r="E12" t="s">
+        <v>13</v>
+      </c>
+      <c r="F12" t="s">
+        <v>75</v>
+      </c>
+      <c r="G12" t="s">
+        <v>15</v>
+      </c>
+      <c r="H12" t="s">
+        <v>16</v>
+      </c>
+      <c r="I12" t="s">
+        <v>76</v>
+      </c>
+      <c r="J12" t="s">
+        <v>77</v>
+      </c>
+      <c r="K12" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>79</v>
+      </c>
+      <c r="B13" t="s">
+        <v>13</v>
+      </c>
+      <c r="C13" t="s">
+        <v>80</v>
+      </c>
+      <c r="D13" t="s">
+        <v>81</v>
+      </c>
+      <c r="E13" t="s">
+        <v>13</v>
+      </c>
+      <c r="F13" t="s">
+        <v>82</v>
+      </c>
+      <c r="G13" t="s">
+        <v>24</v>
+      </c>
+      <c r="H13" t="s">
+        <v>13</v>
+      </c>
+      <c r="I13" t="s">
+        <v>83</v>
+      </c>
+      <c r="J13" t="s">
+        <v>13</v>
+      </c>
+      <c r="K13" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="14" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>85</v>
+      </c>
+      <c r="B14" t="s">
         <v>12</v>
       </c>
-      <c r="D12" t="s">
+      <c r="C14" t="s">
+        <v>13</v>
+      </c>
+      <c r="D14" t="s">
+        <v>13</v>
+      </c>
+      <c r="E14" t="s">
+        <v>13</v>
+      </c>
+      <c r="F14" t="s">
+        <v>86</v>
+      </c>
+      <c r="G14" t="s">
+        <v>15</v>
+      </c>
+      <c r="H14" t="s">
+        <v>87</v>
+      </c>
+      <c r="I14" t="s">
+        <v>88</v>
+      </c>
+      <c r="J14" t="s">
+        <v>89</v>
+      </c>
+      <c r="K14" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="15" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>91</v>
+      </c>
+      <c r="B15" t="s">
         <v>12</v>
       </c>
-      <c r="E12" t="s">
-        <v>12</v>
-      </c>
-      <c r="F12" t="s">
-        <v>73</v>
-      </c>
-      <c r="G12" t="s">
-        <v>22</v>
-      </c>
-      <c r="H12" t="s">
-        <v>69</v>
-      </c>
-      <c r="I12" t="s">
-        <v>74</v>
-      </c>
-      <c r="J12" t="s">
-        <v>75</v>
-      </c>
-      <c r="K12" t="s">
-        <v>76</v>
+      <c r="C15" t="s">
+        <v>13</v>
+      </c>
+      <c r="D15" t="s">
+        <v>13</v>
+      </c>
+      <c r="E15" t="s">
+        <v>13</v>
+      </c>
+      <c r="F15" t="s">
+        <v>92</v>
+      </c>
+      <c r="G15" t="s">
+        <v>15</v>
+      </c>
+      <c r="H15" t="s">
+        <v>87</v>
+      </c>
+      <c r="I15" t="s">
+        <v>93</v>
+      </c>
+      <c r="J15" t="s">
+        <v>94</v>
+      </c>
+      <c r="K15" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="16" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>96</v>
+      </c>
+      <c r="B16" t="s">
+        <v>97</v>
+      </c>
+      <c r="C16" t="s">
+        <v>13</v>
+      </c>
+      <c r="D16" t="s">
+        <v>13</v>
+      </c>
+      <c r="E16" t="s">
+        <v>13</v>
+      </c>
+      <c r="F16" t="s">
+        <v>98</v>
+      </c>
+      <c r="G16" t="s">
+        <v>15</v>
+      </c>
+      <c r="H16" t="s">
+        <v>70</v>
+      </c>
+      <c r="I16" t="s">
+        <v>99</v>
+      </c>
+      <c r="J16" t="s">
+        <v>100</v>
+      </c>
+      <c r="K16" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="17" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>102</v>
+      </c>
+      <c r="B17" t="s">
+        <v>55</v>
+      </c>
+      <c r="C17" t="s">
+        <v>13</v>
+      </c>
+      <c r="D17" t="s">
+        <v>13</v>
+      </c>
+      <c r="E17" t="s">
+        <v>13</v>
+      </c>
+      <c r="F17" t="s">
+        <v>103</v>
+      </c>
+      <c r="G17" t="s">
+        <v>15</v>
+      </c>
+      <c r="H17" t="s">
+        <v>16</v>
+      </c>
+      <c r="I17" t="s">
+        <v>104</v>
+      </c>
+      <c r="J17" t="s">
+        <v>105</v>
+      </c>
+      <c r="K17" t="s">
+        <v>106</v>
       </c>
     </row>
   </sheetData>

</xml_diff>